<commit_message>
ModRank v1.3.0: further architectures, further fusions, and the inflation against a score without information
Adds experiments/20260927-field-inflation: four SurvPath-code-base architectures retrained on the
released folds, three further fitted fusions on all five studies (15 comparisons, none separating),
the inflation D in three studies, and D against a score without information combined by the same
rule (analysis/s33-s35). The README now states that the rank function's tie order depends on the
NumPy build and which builds reproduce the published values to the fourth decimal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014SQjmYtwnex4CpYoifRCbd
</commit_message>
<xml_diff>
--- a/paper/nc-submission/source_data/SourceData.xlsx
+++ b/paper/nc-submission/source_data/SourceData.xlsx
@@ -20254,7 +20254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D135"/>
+  <dimension ref="A1:D175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20731,7 +20731,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SurvPath + clinical/D</t>
+          <t>ModRank/no_signal_D_mean</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -20751,11 +20751,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SurvPath + clinical/ci95[0]</t>
+          <t>ModRank/no_signal_D_central95[0]</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.0196</v>
+        <v>0.0289</v>
       </c>
     </row>
     <row r="28">
@@ -20771,11 +20771,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SurvPath + clinical/ci95[1]</t>
+          <t>ModRank/no_signal_D_central95[1]</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.0668</v>
+        <v>0.0538</v>
       </c>
     </row>
     <row r="29">
@@ -20791,11 +20791,11 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PIBD + clinical/D</t>
+          <t>ModRank/excess_over_no_signal/point</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.0496</v>
+        <v>0.0193</v>
       </c>
     </row>
     <row r="30">
@@ -20811,11 +20811,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PIBD + clinical/ci95[0]</t>
+          <t>ModRank/excess_over_no_signal/mean</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.0238</v>
+        <v>0.0185</v>
       </c>
     </row>
     <row r="31">
@@ -20831,11 +20831,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PIBD + clinical/ci95[1]</t>
+          <t>ModRank/excess_over_no_signal/ci95[0]</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.0769</v>
+        <v>0.0022</v>
       </c>
     </row>
     <row r="32">
@@ -20851,11 +20851,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GSE32894, transcriptome/D</t>
+          <t>ModRank/excess_over_no_signal/ci95[1]</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.0581</v>
+        <v>0.0359</v>
       </c>
     </row>
     <row r="33">
@@ -20871,11 +20871,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GSE32894, transcriptome/ci95[0]</t>
+          <t>ModRank/excess_over_no_signal/p_two_sided</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.0175</v>
+        <v>0.0263</v>
       </c>
     </row>
     <row r="34">
@@ -20891,11 +20891,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GSE32894, transcriptome/ci95[1]</t>
+          <t>SurvPath + clinical/D</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.09710000000000001</v>
+        <v>0.0417</v>
       </c>
     </row>
     <row r="35">
@@ -20911,11 +20911,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GSE31684, transcriptome/D</t>
+          <t>SurvPath + clinical/ci95[0]</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.0253</v>
+        <v>0.0196</v>
       </c>
     </row>
     <row r="36">
@@ -20931,11 +20931,11 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GSE31684, transcriptome/ci95[0]</t>
+          <t>SurvPath + clinical/ci95[1]</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>-0.018</v>
+        <v>0.0668</v>
       </c>
     </row>
     <row r="37">
@@ -20951,17 +20951,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GSE31684, transcriptome/ci95[1]</t>
+          <t>SurvPath + clinical/no_signal_D_mean</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.0678</v>
+        <v>0.0288</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -20971,17 +20971,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ours[0]/quintile</t>
+          <t>SurvPath + clinical/no_signal_D_central95[0]</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -20991,17 +20991,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ours[0]/n</t>
+          <t>SurvPath + clinical/no_signal_D_central95[1]</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>72</v>
+        <v>0.0413</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -21011,17 +21011,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ours[0]/events</t>
+          <t>SurvPath + clinical/excess_over_no_signal/point</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>9</v>
+        <v>0.0129</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -21031,17 +21031,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ours[0]/predicted</t>
+          <t>SurvPath + clinical/excess_over_no_signal/mean</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.1292</v>
+        <v>0.0114</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -21051,17 +21051,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ours[0]/observed_km</t>
+          <t>SurvPath + clinical/excess_over_no_signal/ci95[0]</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.137</v>
+        <v>-0.0035</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -21071,17 +21071,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ours[1]/quintile</t>
+          <t>SurvPath + clinical/excess_over_no_signal/ci95[1]</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -21091,17 +21091,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ours[1]/n</t>
+          <t>SurvPath + clinical/excess_over_no_signal/p_two_sided</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>72</v>
+        <v>0.1373</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -21111,17 +21111,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ours[1]/events</t>
+          <t>PIBD + clinical/D</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>18</v>
+        <v>0.0496</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -21131,17 +21131,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ours[1]/predicted</t>
+          <t>PIBD + clinical/ci95[0]</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.2077</v>
+        <v>0.0238</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -21151,17 +21151,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ours[1]/observed_km</t>
+          <t>PIBD + clinical/ci95[1]</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.2057</v>
+        <v>0.0769</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -21171,17 +21171,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ours[2]/quintile</t>
+          <t>PIBD + clinical/no_signal_D_mean</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>3</v>
+        <v>0.0287</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -21191,17 +21191,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ours[2]/n</t>
+          <t>PIBD + clinical/no_signal_D_central95[0]</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>71</v>
+        <v>0.0154</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -21211,17 +21211,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ours[2]/events</t>
+          <t>PIBD + clinical/no_signal_D_central95[1]</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>18</v>
+        <v>0.0406</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -21231,17 +21231,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ours[2]/predicted</t>
+          <t>PIBD + clinical/excess_over_no_signal/point</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.3099</v>
+        <v>0.021</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -21251,17 +21251,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ours[2]/observed_km</t>
+          <t>PIBD + clinical/excess_over_no_signal/mean</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.2635</v>
+        <v>0.0228</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -21271,17 +21271,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ours[3]/quintile</t>
+          <t>PIBD + clinical/excess_over_no_signal/ci95[0]</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>4</v>
+        <v>0.0066</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -21291,17 +21291,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ours[3]/n</t>
+          <t>PIBD + clinical/excess_over_no_signal/ci95[1]</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>72</v>
+        <v>0.0393</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -21311,17 +21311,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ours[3]/events</t>
+          <t>PIBD + clinical/excess_over_no_signal/p_two_sided</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>30</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -21331,17 +21331,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ours[3]/predicted</t>
+          <t>GSE32894, transcriptome/D</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.4462</v>
+        <v>0.0581</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -21351,17 +21351,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ours[3]/observed_km</t>
+          <t>GSE32894, transcriptome/ci95[0]</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.5085</v>
+        <v>0.0175</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -21371,17 +21371,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ours[4]/quintile</t>
+          <t>GSE32894, transcriptome/ci95[1]</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>5</v>
+        <v>0.09710000000000001</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -21391,17 +21391,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ours[4]/n</t>
+          <t>GSE32894, transcriptome/no_signal_D_mean</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>72</v>
+        <v>0.0183</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -21411,17 +21411,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ours[4]/events</t>
+          <t>GSE32894, transcriptome/no_signal_D_central95[0]</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>38</v>
+        <v>-0.0069</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -21431,17 +21431,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ours[4]/predicted</t>
+          <t>GSE32894, transcriptome/no_signal_D_central95[1]</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.618</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -21451,17 +21451,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ours[4]/observed_km</t>
+          <t>GSE32894, transcriptome/excess_over_no_signal/point</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.6394</v>
+        <v>0.0397</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -21471,17 +21471,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>clinical[0]/quintile</t>
+          <t>GSE32894, transcriptome/excess_over_no_signal/mean</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>0.0409</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -21491,17 +21491,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>clinical[0]/n</t>
+          <t>GSE32894, transcriptome/excess_over_no_signal/ci95[0]</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>72</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -21511,17 +21511,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>clinical[0]/events</t>
+          <t>GSE32894, transcriptome/excess_over_no_signal/ci95[1]</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>16</v>
+        <v>0.0775</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -21531,17 +21531,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>clinical[0]/predicted</t>
+          <t>GSE32894, transcriptome/excess_over_no_signal/p_two_sided</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.1546</v>
+        <v>0.0317</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -21551,17 +21551,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>clinical[0]/observed_km</t>
+          <t>GSE31684, transcriptome/D</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.2168</v>
+        <v>0.0253</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -21571,17 +21571,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>clinical[1]/quintile</t>
+          <t>GSE31684, transcriptome/ci95[0]</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>2</v>
+        <v>-0.018</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -21591,17 +21591,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>clinical[1]/n</t>
+          <t>GSE31684, transcriptome/ci95[1]</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>72</v>
+        <v>0.0678</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -21611,17 +21611,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>clinical[1]/events</t>
+          <t>GSE31684, transcriptome/no_signal_D_mean</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>16</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -21631,17 +21631,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>clinical[1]/predicted</t>
+          <t>GSE31684, transcriptome/no_signal_D_central95[0]</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.2236</v>
+        <v>-0.0148</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -21651,17 +21651,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>clinical[1]/observed_km</t>
+          <t>GSE31684, transcriptome/no_signal_D_central95[1]</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.2395</v>
+        <v>0.0436</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -21671,17 +21671,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>clinical[2]/quintile</t>
+          <t>GSE31684, transcriptome/excess_over_no_signal/point</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>3</v>
+        <v>0.0103</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -21691,17 +21691,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>clinical[2]/n</t>
+          <t>GSE31684, transcriptome/excess_over_no_signal/mean</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>71</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -21711,17 +21711,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>clinical[2]/events</t>
+          <t>GSE31684, transcriptome/excess_over_no_signal/ci95[0]</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>9</v>
+        <v>-0.0325</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -21731,17 +21731,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>clinical[2]/predicted</t>
+          <t>GSE31684, transcriptome/excess_over_no_signal/ci95[1]</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.3132</v>
+        <v>0.0335</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -21751,11 +21751,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>clinical[2]/observed_km</t>
+          <t>GSE31684, transcriptome/excess_over_no_signal/p_two_sided</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.155</v>
+        <v>0.9813</v>
       </c>
     </row>
     <row r="78">
@@ -21771,11 +21771,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>clinical[3]/quintile</t>
+          <t>ours[0]/quintile</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -21791,7 +21791,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>clinical[3]/n</t>
+          <t>ours[0]/n</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -21811,11 +21811,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>clinical[3]/events</t>
+          <t>ours[0]/events</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81">
@@ -21831,11 +21831,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>clinical[3]/predicted</t>
+          <t>ours[0]/predicted</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.4275</v>
+        <v>0.1292</v>
       </c>
     </row>
     <row r="82">
@@ -21851,11 +21851,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>clinical[3]/observed_km</t>
+          <t>ours[0]/observed_km</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.4901</v>
+        <v>0.137</v>
       </c>
     </row>
     <row r="83">
@@ -21871,11 +21871,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>clinical[4]/quintile</t>
+          <t>ours[1]/quintile</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
@@ -21891,7 +21891,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>clinical[4]/n</t>
+          <t>ours[1]/n</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -21911,11 +21911,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>clinical[4]/events</t>
+          <t>ours[1]/events</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
     </row>
     <row r="86">
@@ -21931,11 +21931,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>clinical[4]/predicted</t>
+          <t>ours[1]/predicted</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.5669</v>
+        <v>0.2077</v>
       </c>
     </row>
     <row r="87">
@@ -21951,17 +21951,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>clinical[4]/observed_km</t>
+          <t>ours[1]/observed_km</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.2057</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -21971,17 +21971,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>thresholds[0]</t>
+          <t>ours[2]/quintile</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.05</v>
+        <v>3</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -21991,17 +21991,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>thresholds[1]</t>
+          <t>ours[2]/n</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.1</v>
+        <v>71</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -22011,17 +22011,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>thresholds[2]</t>
+          <t>ours[2]/events</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -22031,17 +22031,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>thresholds[3]</t>
+          <t>ours[2]/predicted</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.2</v>
+        <v>0.3099</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -22051,17 +22051,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>thresholds[4]</t>
+          <t>ours[2]/observed_km</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.25</v>
+        <v>0.2635</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -22071,17 +22071,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>thresholds[5]</t>
+          <t>ours[3]/quintile</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -22091,17 +22091,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>thresholds[6]</t>
+          <t>ours[3]/n</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.35</v>
+        <v>72</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -22111,17 +22111,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>thresholds[7]</t>
+          <t>ours[3]/events</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.4</v>
+        <v>30</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -22131,17 +22131,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>thresholds[8]</t>
+          <t>ours[3]/predicted</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.45</v>
+        <v>0.4462</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -22151,17 +22151,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>thresholds[9]</t>
+          <t>ours[3]/observed_km</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.5</v>
+        <v>0.5085</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -22171,17 +22171,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>thresholds[10]</t>
+          <t>ours[4]/quintile</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.55</v>
+        <v>5</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -22191,17 +22191,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>thresholds[11]</t>
+          <t>ours[4]/n</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.6</v>
+        <v>72</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -22211,17 +22211,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>ModRank[0]</t>
+          <t>ours[4]/events</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.3064</v>
+        <v>38</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -22231,17 +22231,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ModRank[1]</t>
+          <t>ours[4]/predicted</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.2642</v>
+        <v>0.618</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -22251,17 +22251,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ModRank[2]</t>
+          <t>ours[4]/observed_km</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.2209</v>
+        <v>0.6394</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -22271,17 +22271,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ModRank[3]</t>
+          <t>clinical[0]/quintile</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.1785</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -22291,17 +22291,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ModRank[4]</t>
+          <t>clinical[0]/n</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.164</v>
+        <v>72</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -22311,17 +22311,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ModRank[5]</t>
+          <t>clinical[0]/events</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.1444</v>
+        <v>16</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -22331,17 +22331,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ModRank[6]</t>
+          <t>clinical[0]/predicted</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.1222</v>
+        <v>0.1546</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -22351,17 +22351,17 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ModRank[7]</t>
+          <t>clinical[0]/observed_km</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.1356</v>
+        <v>0.2168</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -22371,17 +22371,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>ModRank[8]</t>
+          <t>clinical[1]/quintile</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.093</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -22391,17 +22391,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ModRank[9]</t>
+          <t>clinical[1]/n</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.0712</v>
+        <v>72</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -22411,17 +22411,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ModRank[10]</t>
+          <t>clinical[1]/events</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.0347</v>
+        <v>16</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -22431,17 +22431,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ModRank[11]</t>
+          <t>clinical[1]/predicted</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.0136</v>
+        <v>0.2236</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -22451,17 +22451,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>clinical[0]</t>
+          <t>clinical[1]/observed_km</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.3064</v>
+        <v>0.2395</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -22471,17 +22471,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>clinical[1]</t>
+          <t>clinical[2]/quintile</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.2678</v>
+        <v>3</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -22491,17 +22491,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>clinical[2]</t>
+          <t>clinical[2]/n</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.2147</v>
+        <v>71</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -22511,17 +22511,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>clinical[3]</t>
+          <t>clinical[2]/events</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.1691</v>
+        <v>9</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -22531,17 +22531,17 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>clinical[4]</t>
+          <t>clinical[2]/predicted</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0.13</v>
+        <v>0.3132</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -22551,17 +22551,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>clinical[5]</t>
+          <t>clinical[2]/observed_km</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0.1078</v>
+        <v>0.155</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -22571,17 +22571,17 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>clinical[6]</t>
+          <t>clinical[3]/quintile</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.1054</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -22591,17 +22591,17 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>clinical[7]</t>
+          <t>clinical[3]/n</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.0901</v>
+        <v>72</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -22611,17 +22611,17 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>clinical[8]</t>
+          <t>clinical[3]/events</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>0.0514</v>
+        <v>34</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -22631,17 +22631,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>clinical[9]</t>
+          <t>clinical[3]/predicted</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>0.0227</v>
+        <v>0.4275</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -22651,17 +22651,17 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>clinical[10]</t>
+          <t>clinical[3]/observed_km</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>0.025</v>
+        <v>0.4901</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -22671,17 +22671,17 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>clinical[11]</t>
+          <t>clinical[4]/quintile</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>-0.0117</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -22691,17 +22691,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>treat all[0]</t>
+          <t>clinical[4]/n</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>0.3064</v>
+        <v>72</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -22711,17 +22711,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>treat all[1]</t>
+          <t>clinical[4]/events</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>0.2678</v>
+        <v>38</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -22731,17 +22731,17 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>treat all[2]</t>
+          <t>clinical[4]/predicted</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>0.2248</v>
+        <v>0.5669</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -22751,11 +22751,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>treat all[3]</t>
+          <t>clinical[4]/observed_km</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>0.1763</v>
+        <v>0.5489000000000001</v>
       </c>
     </row>
     <row r="128">
@@ -22771,11 +22771,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>treat all[4]</t>
+          <t>thresholds[0]</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.1214</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="129">
@@ -22791,11 +22791,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>treat all[5]</t>
+          <t>thresholds[1]</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0.0586</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="130">
@@ -22811,11 +22811,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>treat all[6]</t>
+          <t>thresholds[2]</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>-0.0138</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="131">
@@ -22831,11 +22831,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>treat all[7]</t>
+          <t>thresholds[3]</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>-0.0982</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="132">
@@ -22851,11 +22851,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>treat all[8]</t>
+          <t>thresholds[4]</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>-0.1981</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="133">
@@ -22871,11 +22871,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>treat all[9]</t>
+          <t>thresholds[5]</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>-0.3179</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="134">
@@ -22891,11 +22891,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>treat all[10]</t>
+          <t>thresholds[6]</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>-0.4643</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="135">
@@ -22911,10 +22911,810 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
+          <t>thresholds[7]</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>thresholds[8]</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>thresholds[9]</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>thresholds[10]</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>thresholds[11]</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>ModRank[0]</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>0.3064</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>ModRank[1]</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>0.2642</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>ModRank[2]</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>0.2209</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>ModRank[3]</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>0.1785</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>ModRank[4]</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>0.164</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>ModRank[5]</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>0.1444</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>ModRank[6]</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>0.1222</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>ModRank[7]</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>0.1356</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>ModRank[8]</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>0.093</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>ModRank[9]</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>0.0712</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>ModRank[10]</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>0.0347</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>ModRank[11]</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>0.0136</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>clinical[0]</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>0.3064</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>clinical[1]</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>0.2678</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>clinical[2]</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>0.2147</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>clinical[3]</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>0.1691</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>clinical[4]</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>clinical[5]</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>0.1078</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>clinical[6]</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>0.1054</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>clinical[7]</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>0.0901</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>clinical[8]</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>0.0514</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>clinical[9]</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>0.0227</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>clinical[10]</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>clinical[11]</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>-0.0117</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>treat all[0]</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>0.3064</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>treat all[1]</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>0.2678</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>treat all[2]</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>0.2248</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>treat all[3]</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>0.1763</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>treat all[4]</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>0.1214</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>treat all[5]</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>0.0586</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>treat all[6]</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>-0.0138</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>treat all[7]</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>-0.0982</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>treat all[8]</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>-0.1981</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>treat all[9]</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>-0.3179</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>treat all[10]</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>-0.4643</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>paper/figures/fig7_added_value_utility.source.json</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
           <t>treat all[11]</t>
         </is>
       </c>
-      <c r="D135" t="n">
+      <c r="D175" t="n">
         <v>-0.6474</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ModRank v1.3.2: amendment A2, Breslow risk sets and average ranks, every post-freeze result regenerated
The Cox fit now gives every event the full risk set of its tied time, and tied scores share their
average rank. Every result after the confirmatory run was regenerated (primary 0.7212 -> 0.7214);
experiments/20260928-amendment-a2 holds the protocol, the reproduction of every committed file
under the original functions, and the before-after table. Adds the tuned-ridge stacking
comparator, the figures and .aux files the number gate reads, and one trainer printout per
competitor, so paper/check_numbers.py runs to completion from this repository. The retired BiB
manuscript files are removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper/nc-submission/source_data/SourceData.xlsx
+++ b/paper/nc-submission/source_data/SourceData.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.6637999999999999</v>
+        <v>0.6637</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.5666</v>
+        <v>0.5664</v>
       </c>
     </row>
     <row r="7">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.6596</v>
+        <v>0.6595</v>
       </c>
     </row>
     <row r="9">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.651</v>
+        <v>0.6512</v>
       </c>
     </row>
     <row r="10">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.7225</v>
+        <v>0.7224</v>
       </c>
     </row>
     <row r="11">
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.6856</v>
+        <v>0.6870000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.681</v>
+        <v>0.6805</v>
       </c>
     </row>
     <row r="13">
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.5658</v>
+        <v>0.5642</v>
       </c>
     </row>
     <row r="67">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.6218</v>
+        <v>0.6219</v>
       </c>
     </row>
     <row r="68">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.056</v>
+        <v>0.0577</v>
       </c>
     </row>
     <row r="69">
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>0.5636</v>
+        <v>0.5616</v>
       </c>
     </row>
     <row r="239">
@@ -7421,7 +7421,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>0.5658</v>
+        <v>0.5642</v>
       </c>
     </row>
     <row r="240">
@@ -7441,7 +7441,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>0.6218</v>
+        <v>0.6219</v>
       </c>
     </row>
     <row r="241">
@@ -7461,7 +7461,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>0.6596</v>
+        <v>0.6595</v>
       </c>
     </row>
     <row r="242">
@@ -7481,7 +7481,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>0.651</v>
+        <v>0.6512</v>
       </c>
     </row>
     <row r="243">
@@ -7501,7 +7501,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>0.6841</v>
+        <v>0.6835</v>
       </c>
     </row>
     <row r="244">
@@ -7521,7 +7521,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>0.6992</v>
+        <v>0.7003</v>
       </c>
     </row>
     <row r="245">
@@ -7541,7 +7541,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>0.6861</v>
+        <v>0.6859</v>
       </c>
     </row>
     <row r="246">
@@ -7665,7 +7665,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>-0.0042</v>
+        <v>-0.0058</v>
       </c>
     </row>
     <row r="252">
@@ -7685,7 +7685,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>0.056</v>
+        <v>0.0577</v>
       </c>
     </row>
     <row r="253">
@@ -7875,7 +7875,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>0.4828</v>
+        <v>0.4853</v>
       </c>
     </row>
     <row r="262">
@@ -7895,7 +7895,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>0.4828</v>
+        <v>0.4853</v>
       </c>
     </row>
     <row r="263">
@@ -7915,7 +7915,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>0.5686</v>
+        <v>0.5683</v>
       </c>
     </row>
     <row r="264">
@@ -7935,7 +7935,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>0.7442</v>
+        <v>0.7443</v>
       </c>
     </row>
     <row r="265">
@@ -7955,7 +7955,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>0.5829</v>
+        <v>0.5833</v>
       </c>
     </row>
     <row r="266">
@@ -7975,7 +7975,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>0.7101</v>
+        <v>0.711</v>
       </c>
     </row>
     <row r="267">
@@ -7995,7 +7995,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>0.6892</v>
+        <v>0.6881</v>
       </c>
     </row>
     <row r="268">
@@ -8015,7 +8015,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>0.6614</v>
+        <v>0.6637999999999999</v>
       </c>
     </row>
     <row r="269">
@@ -8139,7 +8139,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>-0.08019999999999999</v>
+        <v>-0.07770000000000001</v>
       </c>
     </row>
     <row r="275">
@@ -8159,7 +8159,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>0.0858</v>
+        <v>0.083</v>
       </c>
     </row>
     <row r="276">
@@ -8349,7 +8349,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>0.469</v>
+        <v>0.4691</v>
       </c>
     </row>
     <row r="285">
@@ -8369,7 +8369,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>0.469</v>
+        <v>0.4691</v>
       </c>
     </row>
     <row r="286">
@@ -8389,7 +8389,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>0.6898</v>
+        <v>0.6902</v>
       </c>
     </row>
     <row r="287">
@@ -8429,7 +8429,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>0.6116</v>
+        <v>0.6117</v>
       </c>
     </row>
     <row r="289">
@@ -8449,7 +8449,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>0.6819</v>
+        <v>0.6825</v>
       </c>
     </row>
     <row r="290">
@@ -8469,7 +8469,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>0.7141</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="291">
@@ -8489,7 +8489,7 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>0.6231</v>
+        <v>0.6247</v>
       </c>
     </row>
     <row r="292">
@@ -8613,7 +8613,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>-0.186</v>
+        <v>-0.1859</v>
       </c>
     </row>
     <row r="298">
@@ -8633,7 +8633,7 @@
         </is>
       </c>
       <c r="D298" t="n">
-        <v>0.2208</v>
+        <v>0.2211</v>
       </c>
     </row>
     <row r="299">
@@ -8933,7 +8933,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>0.485</v>
+        <v>0.4846</v>
       </c>
     </row>
     <row r="313">
@@ -8953,7 +8953,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>0.5027</v>
+        <v>0.5042</v>
       </c>
     </row>
     <row r="314">
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>0.6135</v>
+        <v>0.6133</v>
       </c>
     </row>
     <row r="316">
@@ -9013,7 +9013,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5848</v>
       </c>
     </row>
     <row r="317">
@@ -9033,7 +9033,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>0.6169</v>
+        <v>0.616</v>
       </c>
     </row>
     <row r="318">
@@ -9073,7 +9073,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>0.6015</v>
+        <v>0.6008</v>
       </c>
     </row>
     <row r="320">
@@ -9197,7 +9197,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>-0.009299999999999999</v>
+        <v>-0.0078</v>
       </c>
     </row>
     <row r="326">
@@ -9217,7 +9217,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>0.0423</v>
+        <v>0.0408</v>
       </c>
     </row>
     <row r="327">
@@ -9473,7 +9473,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>0.515</v>
+        <v>0.5153</v>
       </c>
     </row>
     <row r="339">
@@ -9493,7 +9493,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>0.5358000000000001</v>
+        <v>0.5364</v>
       </c>
     </row>
     <row r="340">
@@ -9513,7 +9513,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>0.5819</v>
+        <v>0.5841</v>
       </c>
     </row>
     <row r="341">
@@ -9533,7 +9533,7 @@
         </is>
       </c>
       <c r="D341" t="n">
-        <v>0.5858</v>
+        <v>0.5854</v>
       </c>
     </row>
     <row r="342">
@@ -9593,7 +9593,7 @@
         </is>
       </c>
       <c r="D344" t="n">
-        <v>0.6311</v>
+        <v>0.629</v>
       </c>
     </row>
     <row r="345">
@@ -9613,7 +9613,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>0.6125</v>
+        <v>0.613</v>
       </c>
     </row>
     <row r="346">
@@ -9737,7 +9737,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>-0.0562</v>
+        <v>-0.0556</v>
       </c>
     </row>
     <row r="352">
@@ -9757,7 +9757,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>0.0461</v>
+        <v>0.0477</v>
       </c>
     </row>
     <row r="353">
@@ -10097,7 +10097,7 @@
         </is>
       </c>
       <c r="D369" t="n">
-        <v>0.5658</v>
+        <v>0.5642</v>
       </c>
     </row>
     <row r="370">
@@ -10117,7 +10117,7 @@
         </is>
       </c>
       <c r="D370" t="n">
-        <v>0.6218</v>
+        <v>0.6219</v>
       </c>
     </row>
     <row r="371">
@@ -10137,7 +10137,7 @@
         </is>
       </c>
       <c r="D371" t="n">
-        <v>0.056</v>
+        <v>0.0577</v>
       </c>
     </row>
     <row r="372">
@@ -10374,7 +10374,7 @@
         </is>
       </c>
       <c r="D383" t="n">
-        <v>0.4828</v>
+        <v>0.4853</v>
       </c>
     </row>
     <row r="384">
@@ -10394,7 +10394,7 @@
         </is>
       </c>
       <c r="D384" t="n">
-        <v>0.5686</v>
+        <v>0.5683</v>
       </c>
     </row>
     <row r="385">
@@ -10414,7 +10414,7 @@
         </is>
       </c>
       <c r="D385" t="n">
-        <v>0.0858</v>
+        <v>0.083</v>
       </c>
     </row>
     <row r="386">
@@ -10651,7 +10651,7 @@
         </is>
       </c>
       <c r="D397" t="n">
-        <v>0.469</v>
+        <v>0.4691</v>
       </c>
     </row>
     <row r="398">
@@ -10671,7 +10671,7 @@
         </is>
       </c>
       <c r="D398" t="n">
-        <v>0.6898</v>
+        <v>0.6902</v>
       </c>
     </row>
     <row r="399">
@@ -10691,7 +10691,7 @@
         </is>
       </c>
       <c r="D399" t="n">
-        <v>0.2208</v>
+        <v>0.2211</v>
       </c>
     </row>
     <row r="400">
@@ -11091,7 +11091,7 @@
         </is>
       </c>
       <c r="D419" t="n">
-        <v>0.5027</v>
+        <v>0.5042</v>
       </c>
     </row>
     <row r="420">
@@ -11131,7 +11131,7 @@
         </is>
       </c>
       <c r="D421" t="n">
-        <v>0.0423</v>
+        <v>0.0408</v>
       </c>
     </row>
     <row r="422">
@@ -11491,7 +11491,7 @@
         </is>
       </c>
       <c r="D439" t="n">
-        <v>0.5358000000000001</v>
+        <v>0.5364</v>
       </c>
     </row>
     <row r="440">
@@ -11511,7 +11511,7 @@
         </is>
       </c>
       <c r="D440" t="n">
-        <v>0.5819</v>
+        <v>0.5841</v>
       </c>
     </row>
     <row r="441">
@@ -11531,7 +11531,7 @@
         </is>
       </c>
       <c r="D441" t="n">
-        <v>0.0461</v>
+        <v>0.0477</v>
       </c>
     </row>
     <row r="442">
@@ -11613,7 +11613,7 @@
         </is>
       </c>
       <c r="D445" t="n">
-        <v>0.7291</v>
+        <v>0.7287</v>
       </c>
     </row>
     <row r="446">
@@ -11755,7 +11755,7 @@
         </is>
       </c>
       <c r="D452" t="n">
-        <v>0.6637999999999999</v>
+        <v>0.6637</v>
       </c>
     </row>
     <row r="453">
@@ -11775,7 +11775,7 @@
         </is>
       </c>
       <c r="D453" t="n">
-        <v>0.7225</v>
+        <v>0.7224</v>
       </c>
     </row>
     <row r="454">
@@ -11835,7 +11835,7 @@
         </is>
       </c>
       <c r="D456" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="457">
@@ -11917,7 +11917,7 @@
         </is>
       </c>
       <c r="D460" t="n">
-        <v>0.5666</v>
+        <v>0.5664</v>
       </c>
     </row>
     <row r="461">
@@ -11937,7 +11937,7 @@
         </is>
       </c>
       <c r="D461" t="n">
-        <v>0.6856</v>
+        <v>0.6870000000000001</v>
       </c>
     </row>
     <row r="462">
@@ -11997,7 +11997,7 @@
         </is>
       </c>
       <c r="D464" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="465">
@@ -12239,7 +12239,7 @@
         </is>
       </c>
       <c r="D476" t="n">
-        <v>0.6997</v>
+        <v>0.6983</v>
       </c>
     </row>
     <row r="477">
@@ -12399,7 +12399,7 @@
         </is>
       </c>
       <c r="D484" t="n">
-        <v>0.6693</v>
+        <v>0.669</v>
       </c>
     </row>
     <row r="485">
@@ -12419,7 +12419,7 @@
         </is>
       </c>
       <c r="D485" t="n">
-        <v>0.6226</v>
+        <v>0.6232</v>
       </c>
     </row>
     <row r="486">
@@ -13882,7 +13882,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.021</v>
+        <v>0.0211</v>
       </c>
     </row>
     <row r="73">
@@ -13902,7 +13902,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.0589</v>
+        <v>0.059</v>
       </c>
     </row>
     <row r="74">
@@ -13922,7 +13922,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.355</v>
+        <v>0.352</v>
       </c>
     </row>
     <row r="75">
@@ -14026,7 +14026,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.7237</v>
+        <v>0.7233000000000001</v>
       </c>
     </row>
     <row r="80">
@@ -14066,7 +14066,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.6647999999999999</v>
+        <v>0.6637</v>
       </c>
     </row>
     <row r="82">
@@ -14086,7 +14086,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.6644</v>
+        <v>0.6645</v>
       </c>
     </row>
     <row r="83">
@@ -14106,7 +14106,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.6897</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="84">
@@ -14126,7 +14126,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.6897</v>
+        <v>0.6894</v>
       </c>
     </row>
     <row r="85">
@@ -14146,7 +14146,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0.6989</v>
+        <v>0.6982</v>
       </c>
     </row>
     <row r="86">
@@ -14166,7 +14166,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.6639</v>
+        <v>0.6643</v>
       </c>
     </row>
     <row r="87">
@@ -14328,7 +14328,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.6989</v>
+        <v>0.6982</v>
       </c>
     </row>
     <row r="95">
@@ -14348,7 +14348,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.781</v>
+        <v>0.7794</v>
       </c>
     </row>
     <row r="96">
@@ -14368,7 +14368,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.7516</v>
+        <v>0.7504999999999999</v>
       </c>
     </row>
     <row r="97">
@@ -14388,7 +14388,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.7385</v>
+        <v>0.7372</v>
       </c>
     </row>
     <row r="98">
@@ -14408,7 +14408,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.195</v>
+        <v>0.1951</v>
       </c>
     </row>
     <row r="99">
@@ -14428,7 +14428,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>4.3e-09</v>
+        <v>8.63e-09</v>
       </c>
     </row>
     <row r="100">
@@ -14708,7 +14708,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.6639</v>
+        <v>0.6643</v>
       </c>
     </row>
     <row r="114">
@@ -14728,7 +14728,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.7039</v>
+        <v>0.7054</v>
       </c>
     </row>
     <row r="115">
@@ -14748,7 +14748,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.6988</v>
+        <v>0.7008</v>
       </c>
     </row>
     <row r="116">
@@ -14768,7 +14768,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0.7027</v>
+        <v>0.7028</v>
       </c>
     </row>
     <row r="117">
@@ -14808,7 +14808,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>9.380000000000001e-08</v>
+        <v>6.5e-08</v>
       </c>
     </row>
     <row r="119">
@@ -15023,7 +15023,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.0588</v>
+        <v>0.0595</v>
       </c>
     </row>
     <row r="6">
@@ -15043,7 +15043,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.0172</v>
+        <v>0.0174</v>
       </c>
     </row>
     <row r="7">
@@ -15063,7 +15063,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.1009</v>
+        <v>0.1025</v>
       </c>
     </row>
     <row r="8">
@@ -15083,7 +15083,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.0053</v>
+        <v>0.0057</v>
       </c>
     </row>
     <row r="9">
@@ -15103,7 +15103,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.0265</v>
+        <v>0.0285</v>
       </c>
     </row>
     <row r="10">
@@ -15143,7 +15143,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.0704</v>
+        <v>0.0699</v>
       </c>
     </row>
     <row r="12">
@@ -15163,7 +15163,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.0288</v>
+        <v>0.0279</v>
       </c>
     </row>
     <row r="13">
@@ -15183,7 +15183,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.1138</v>
+        <v>0.1136</v>
       </c>
     </row>
     <row r="14">
@@ -15263,7 +15263,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.0594</v>
+        <v>0.0587</v>
       </c>
     </row>
     <row r="18">
@@ -15283,7 +15283,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.0111</v>
+        <v>0.0107</v>
       </c>
     </row>
     <row r="19">
@@ -15303,7 +15303,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.107</v>
+        <v>0.1065</v>
       </c>
     </row>
     <row r="20">
@@ -15323,7 +15323,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.0163</v>
+        <v>0.0167</v>
       </c>
     </row>
     <row r="21">
@@ -15343,7 +15343,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0668</v>
       </c>
     </row>
     <row r="22">
@@ -15383,7 +15383,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.034</v>
+        <v>0.0333</v>
       </c>
     </row>
     <row r="24">
@@ -15403,7 +15403,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.005</v>
+        <v>0.0041</v>
       </c>
     </row>
     <row r="25">
@@ -15423,7 +15423,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.0635</v>
+        <v>0.063</v>
       </c>
     </row>
     <row r="26">
@@ -15443,7 +15443,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.0187</v>
+        <v>0.0243</v>
       </c>
     </row>
     <row r="27">
@@ -15463,7 +15463,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.07290000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -15503,7 +15503,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.034</v>
+        <v>0.0338</v>
       </c>
     </row>
     <row r="30">
@@ -15523,7 +15523,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>-0.0056</v>
+        <v>-0.0053</v>
       </c>
     </row>
     <row r="31">
@@ -15543,7 +15543,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.0731</v>
+        <v>0.0727</v>
       </c>
     </row>
     <row r="32">
@@ -15563,7 +15563,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.0843</v>
+        <v>0.0867</v>
       </c>
     </row>
     <row r="33">
@@ -15583,7 +15583,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.1686</v>
+        <v>0.1734</v>
       </c>
     </row>
     <row r="34">
@@ -15623,7 +15623,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.0249</v>
+        <v>0.0252</v>
       </c>
     </row>
     <row r="36">
@@ -15643,7 +15643,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>-0.0181</v>
+        <v>-0.0173</v>
       </c>
     </row>
     <row r="37">
@@ -15663,7 +15663,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.0675</v>
+        <v>0.06759999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -15683,7 +15683,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.2413</v>
+        <v>0.2383</v>
       </c>
     </row>
     <row r="39">
@@ -15703,7 +15703,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.2413</v>
+        <v>0.2383</v>
       </c>
     </row>
     <row r="40">
@@ -15743,7 +15743,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.6596</v>
+        <v>0.6595</v>
       </c>
     </row>
     <row r="42">
@@ -15763,7 +15763,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.651</v>
+        <v>0.6512</v>
       </c>
     </row>
     <row r="43">
@@ -15783,7 +15783,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.6637999999999999</v>
+        <v>0.6637</v>
       </c>
     </row>
     <row r="44">
@@ -15803,7 +15803,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.6841</v>
+        <v>0.6835</v>
       </c>
     </row>
     <row r="45">
@@ -15823,7 +15823,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.7</v>
+        <v>0.6997</v>
       </c>
     </row>
     <row r="46">
@@ -15843,7 +15843,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.7005</v>
+        <v>0.7002</v>
       </c>
     </row>
     <row r="47">
@@ -15863,7 +15863,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.7225</v>
+        <v>0.7224</v>
       </c>
     </row>
     <row r="48">
@@ -15883,7 +15883,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>-0.022</v>
+        <v>-0.0222</v>
       </c>
     </row>
     <row r="49">
@@ -15903,7 +15903,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>-0.0225</v>
+        <v>-0.0227</v>
       </c>
     </row>
     <row r="50">
@@ -15923,7 +15923,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>-0.0384</v>
+        <v>-0.0389</v>
       </c>
     </row>
     <row r="51">
@@ -15943,7 +15943,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>-0.0218</v>
+        <v>-0.0221</v>
       </c>
     </row>
     <row r="52">
@@ -15983,7 +15983,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-0.0481</v>
+        <v>-0.0484</v>
       </c>
     </row>
     <row r="54">
@@ -16003,7 +16003,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.0038</v>
+        <v>0.0039</v>
       </c>
     </row>
     <row r="55">
@@ -16023,7 +16023,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.1047</v>
+        <v>0.09669999999999999</v>
       </c>
     </row>
     <row r="56">
@@ -16043,7 +16043,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>-0.0222</v>
+        <v>-0.0224</v>
       </c>
     </row>
     <row r="57">
@@ -16083,7 +16083,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>-0.0489</v>
+        <v>-0.0495</v>
       </c>
     </row>
     <row r="59">
@@ -16103,7 +16103,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.006</v>
+        <v>0.0055</v>
       </c>
     </row>
     <row r="60">
@@ -16123,7 +16123,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.11</v>
+        <v>0.1073</v>
       </c>
     </row>
     <row r="61">
@@ -16143,7 +16143,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>-0.0385</v>
+        <v>-0.039</v>
       </c>
     </row>
     <row r="62">
@@ -16163,7 +16163,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.0154</v>
+        <v>0.0156</v>
       </c>
     </row>
     <row r="63">
@@ -16183,7 +16183,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>-0.0687</v>
+        <v>-0.0696</v>
       </c>
     </row>
     <row r="64">
@@ -16203,7 +16203,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.0086</v>
       </c>
     </row>
     <row r="65">
@@ -16223,7 +16223,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.01</v>
+        <v>0.0107</v>
       </c>
     </row>
     <row r="66">
@@ -16678,7 +16678,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.7225</v>
+        <v>0.7224</v>
       </c>
     </row>
     <row r="6">
@@ -16698,7 +16698,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.7248</v>
+        <v>0.7247</v>
       </c>
     </row>
     <row r="7">
@@ -16718,7 +16718,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.7129</v>
+        <v>0.7143</v>
       </c>
     </row>
     <row r="8">
@@ -16738,7 +16738,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.7243000000000001</v>
+        <v>0.7247</v>
       </c>
     </row>
     <row r="9">
@@ -16758,7 +16758,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.7216</v>
+        <v>0.721</v>
       </c>
     </row>
     <row r="10">
@@ -16778,7 +16778,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.7131999999999999</v>
+        <v>0.7137</v>
       </c>
     </row>
     <row r="11">
@@ -16798,7 +16798,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.7111</v>
+        <v>0.7118</v>
       </c>
     </row>
     <row r="12">
@@ -16818,7 +16818,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.7030999999999999</v>
+        <v>0.7056</v>
       </c>
     </row>
     <row r="13">
@@ -16838,7 +16838,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.7108</v>
+        <v>0.7128</v>
       </c>
     </row>
     <row r="14">
@@ -16858,7 +16858,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.7146</v>
+        <v>0.7098</v>
       </c>
     </row>
     <row r="15">
@@ -16878,7 +16878,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.6907</v>
       </c>
     </row>
     <row r="16">
@@ -16898,7 +16898,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.6798999999999999</v>
+        <v>0.6797</v>
       </c>
     </row>
     <row r="17">
@@ -16918,7 +16918,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.6907</v>
       </c>
     </row>
     <row r="18">
@@ -16938,7 +16938,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.6907</v>
       </c>
     </row>
     <row r="19">
@@ -16958,7 +16958,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.679</v>
+        <v>0.6785</v>
       </c>
     </row>
     <row r="20">
@@ -16998,7 +16998,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.7252999999999999</v>
+        <v>0.7243000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -17018,7 +17018,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.7153</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="23">
@@ -17038,7 +17038,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.7067</v>
+        <v>0.7066</v>
       </c>
     </row>
     <row r="24">
@@ -17058,7 +17058,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.7028</v>
+        <v>0.702</v>
       </c>
     </row>
     <row r="25">
@@ -17078,7 +17078,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.7247</v>
+        <v>0.7242</v>
       </c>
     </row>
     <row r="26">
@@ -17098,7 +17098,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.7114</v>
+        <v>0.7089</v>
       </c>
     </row>
     <row r="27">
@@ -17118,7 +17118,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.7288</v>
+        <v>0.7282999999999999</v>
       </c>
     </row>
     <row r="28">
@@ -17138,7 +17138,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.698</v>
+        <v>0.6987</v>
       </c>
     </row>
     <row r="29">
@@ -17158,7 +17158,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.7229</v>
+        <v>0.7247</v>
       </c>
     </row>
     <row r="30">
@@ -17178,7 +17178,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.7174</v>
+        <v>0.7171</v>
       </c>
     </row>
     <row r="31">
@@ -17198,7 +17198,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.7161</v>
+        <v>0.7166</v>
       </c>
     </row>
     <row r="32">
@@ -17218,7 +17218,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.7227</v>
+        <v>0.722</v>
       </c>
     </row>
     <row r="33">
@@ -17238,7 +17238,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.7145</v>
+        <v>0.7157</v>
       </c>
     </row>
     <row r="34">
@@ -17258,7 +17258,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.7091</v>
+        <v>0.7094</v>
       </c>
     </row>
     <row r="35">
@@ -17278,7 +17278,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.7323</v>
+        <v>0.7322</v>
       </c>
     </row>
     <row r="36">
@@ -17298,7 +17298,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.7163</v>
+        <v>0.7164</v>
       </c>
     </row>
     <row r="37">
@@ -17318,7 +17318,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.714</v>
+        <v>0.7124</v>
       </c>
     </row>
     <row r="38">
@@ -17338,7 +17338,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.7164</v>
+        <v>0.7161</v>
       </c>
     </row>
     <row r="39">
@@ -17358,7 +17358,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.7212</v>
+        <v>0.7216</v>
       </c>
     </row>
     <row r="40">
@@ -17378,7 +17378,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.7104</v>
+        <v>0.7106</v>
       </c>
     </row>
     <row r="41">
@@ -17398,7 +17398,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.711</v>
+        <v>0.7123</v>
       </c>
     </row>
     <row r="42">
@@ -17418,7 +17418,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.7076</v>
+        <v>0.7074</v>
       </c>
     </row>
     <row r="43">
@@ -17438,7 +17438,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.7291</v>
+        <v>0.7285</v>
       </c>
     </row>
     <row r="44">
@@ -17458,7 +17458,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.6957</v>
+        <v>0.6947</v>
       </c>
     </row>
     <row r="45">
@@ -17478,7 +17478,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.7066</v>
+        <v>0.7081</v>
       </c>
     </row>
     <row r="46">
@@ -17498,7 +17498,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.6881</v>
+        <v>0.6879999999999999</v>
       </c>
     </row>
     <row r="47">
@@ -17518,7 +17518,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.7015</v>
+        <v>0.7008</v>
       </c>
     </row>
     <row r="48">
@@ -17538,7 +17538,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.6897</v>
+        <v>0.6921</v>
       </c>
     </row>
     <row r="49">
@@ -17558,7 +17558,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.7211</v>
+        <v>0.7208</v>
       </c>
     </row>
     <row r="50">
@@ -17578,7 +17578,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.7042</v>
+        <v>0.7043</v>
       </c>
     </row>
     <row r="51">
@@ -17598,7 +17598,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.7147</v>
+        <v>0.7156</v>
       </c>
     </row>
     <row r="52">
@@ -17618,7 +17618,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.6916</v>
+        <v>0.6928</v>
       </c>
     </row>
     <row r="53">
@@ -17638,7 +17638,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.7181999999999999</v>
+        <v>0.7201</v>
       </c>
     </row>
     <row r="54">
@@ -17658,7 +17658,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.7137</v>
+        <v>0.7134</v>
       </c>
     </row>
     <row r="55">
@@ -17678,7 +17678,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.6952</v>
+        <v>0.6948</v>
       </c>
     </row>
     <row r="56">
@@ -17698,7 +17698,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.7053</v>
+        <v>0.7047</v>
       </c>
     </row>
     <row r="57">
@@ -17718,7 +17718,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.7107</v>
+        <v>0.7094</v>
       </c>
     </row>
     <row r="58">
@@ -17738,7 +17738,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.6952</v>
+        <v>0.6967</v>
       </c>
     </row>
     <row r="59">
@@ -17758,7 +17758,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.7131999999999999</v>
+        <v>0.7133</v>
       </c>
     </row>
     <row r="60">
@@ -17778,7 +17778,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.6997</v>
+        <v>0.7002</v>
       </c>
     </row>
     <row r="61">
@@ -17798,7 +17798,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.7093</v>
+        <v>0.709</v>
       </c>
     </row>
     <row r="62">
@@ -17818,7 +17818,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.7122000000000001</v>
+        <v>0.7119</v>
       </c>
     </row>
     <row r="63">
@@ -17838,7 +17838,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.7078</v>
+        <v>0.7091</v>
       </c>
     </row>
     <row r="64">
@@ -17858,7 +17858,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.6984</v>
+        <v>0.6982</v>
       </c>
     </row>
     <row r="65">
@@ -17878,7 +17878,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.7022</v>
+        <v>0.7024</v>
       </c>
     </row>
     <row r="66">
@@ -17898,7 +17898,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.6959</v>
+        <v>0.6966</v>
       </c>
     </row>
     <row r="67">
@@ -17918,7 +17918,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.721</v>
+        <v>0.7205</v>
       </c>
     </row>
     <row r="68">
@@ -17938,7 +17938,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.6656</v>
+        <v>0.6657</v>
       </c>
     </row>
     <row r="69">
@@ -17958,7 +17958,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.6848</v>
+        <v>0.6849</v>
       </c>
     </row>
     <row r="70">
@@ -17978,7 +17978,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.6888</v>
+        <v>0.6884</v>
       </c>
     </row>
     <row r="71">
@@ -17998,7 +17998,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.6623</v>
+        <v>0.644</v>
       </c>
     </row>
     <row r="72">
@@ -18018,7 +18018,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.674</v>
+        <v>0.6665</v>
       </c>
     </row>
     <row r="73">
@@ -18038,7 +18038,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.6633</v>
+        <v>0.6634</v>
       </c>
     </row>
     <row r="74">
@@ -18058,7 +18058,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.6674</v>
+        <v>0.6676</v>
       </c>
     </row>
     <row r="75">
@@ -18078,7 +18078,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.6898</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="76">
@@ -18098,7 +18098,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.6666</v>
+        <v>0.6669</v>
       </c>
     </row>
     <row r="77">
@@ -18138,7 +18138,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.6504</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="79">
@@ -18158,7 +18158,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.6802</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="80">
@@ -18198,7 +18198,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.6633</v>
+        <v>0.6627</v>
       </c>
     </row>
     <row r="82">
@@ -18218,7 +18218,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.648</v>
+        <v>0.647</v>
       </c>
     </row>
     <row r="83">
@@ -18238,7 +18238,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.6908</v>
+        <v>0.6907</v>
       </c>
     </row>
     <row r="84">
@@ -18258,7 +18258,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.6877</v>
+        <v>0.6879999999999999</v>
       </c>
     </row>
     <row r="85">
@@ -18318,7 +18318,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.6356000000000001</v>
+        <v>0.644</v>
       </c>
     </row>
     <row r="88">
@@ -18338,7 +18338,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.6758</v>
+        <v>0.6754</v>
       </c>
     </row>
     <row r="89">
@@ -18358,7 +18358,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.6591</v>
+        <v>0.6594</v>
       </c>
     </row>
     <row r="90">
@@ -18378,7 +18378,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.6843</v>
+        <v>0.6837</v>
       </c>
     </row>
     <row r="91">
@@ -18398,7 +18398,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.6783</v>
+        <v>0.6784</v>
       </c>
     </row>
     <row r="92">
@@ -18418,7 +18418,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.6525</v>
+        <v>0.6523</v>
       </c>
     </row>
     <row r="93">
@@ -18438,7 +18438,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.6586</v>
+        <v>0.6585</v>
       </c>
     </row>
     <row r="94">
@@ -18518,7 +18518,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.6684</v>
+        <v>0.6685</v>
       </c>
     </row>
     <row r="98">
@@ -18538,7 +18538,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.6612</v>
+        <v>0.6611</v>
       </c>
     </row>
     <row r="99">
@@ -18558,7 +18558,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.6736</v>
+        <v>0.6731</v>
       </c>
     </row>
     <row r="100">
@@ -18578,7 +18578,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.6618000000000001</v>
+        <v>0.6617</v>
       </c>
     </row>
     <row r="101">
@@ -18598,7 +18598,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.6633</v>
+        <v>0.6631</v>
       </c>
     </row>
     <row r="102">
@@ -18618,7 +18618,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.6646</v>
+        <v>0.664</v>
       </c>
     </row>
     <row r="103">
@@ -18638,7 +18638,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.6615</v>
+        <v>0.6614</v>
       </c>
     </row>
     <row r="104">
@@ -18678,7 +18678,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.6555</v>
+        <v>0.6553</v>
       </c>
     </row>
     <row r="106">
@@ -18718,7 +18718,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.665</v>
+        <v>0.6653</v>
       </c>
     </row>
     <row r="108">
@@ -18738,7 +18738,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.661</v>
+        <v>0.6608000000000001</v>
       </c>
     </row>
     <row r="109">
@@ -18758,7 +18758,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.6608000000000001</v>
+        <v>0.6597</v>
       </c>
     </row>
     <row r="110">
@@ -18778,7 +18778,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.6618000000000001</v>
+        <v>0.6616</v>
       </c>
     </row>
     <row r="111">
@@ -18798,7 +18798,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.6593</v>
+        <v>0.6594</v>
       </c>
     </row>
     <row r="112">
@@ -18818,7 +18818,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.6425</v>
+        <v>0.642</v>
       </c>
     </row>
     <row r="113">
@@ -18838,7 +18838,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.6677</v>
+        <v>0.6673</v>
       </c>
     </row>
     <row r="114">
@@ -19138,7 +19138,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.6989</v>
+        <v>0.6964</v>
       </c>
     </row>
     <row r="129">
@@ -19158,7 +19158,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0.7196</v>
+        <v>0.7187</v>
       </c>
     </row>
     <row r="130">
@@ -19178,7 +19178,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>0.7196</v>
+        <v>0.7226</v>
       </c>
     </row>
     <row r="131">
@@ -19258,7 +19258,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.5272</v>
+        <v>0.5256</v>
       </c>
     </row>
     <row r="135">
@@ -19338,7 +19338,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.7010999999999999</v>
+        <v>0.7023</v>
       </c>
     </row>
     <row r="139">
@@ -19358,7 +19358,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.639</v>
+        <v>0.6394</v>
       </c>
     </row>
     <row r="140">
@@ -19478,7 +19478,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>0.6443</v>
+        <v>0.6432</v>
       </c>
     </row>
     <row r="146">
@@ -19558,7 +19558,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0.7038</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="150">
@@ -19578,7 +19578,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0.6584</v>
+        <v>0.6573</v>
       </c>
     </row>
     <row r="151">
@@ -19598,7 +19598,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>0.627</v>
+        <v>0.6259</v>
       </c>
     </row>
     <row r="152">
@@ -19618,7 +19618,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>0.6584</v>
+        <v>0.6573</v>
       </c>
     </row>
     <row r="153">
@@ -19758,7 +19758,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>0.5746</v>
+        <v>0.5731000000000001</v>
       </c>
     </row>
     <row r="160">
@@ -19778,7 +19778,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>0.7231</v>
+        <v>0.7235</v>
       </c>
     </row>
     <row r="161">
@@ -19798,7 +19798,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0.7007</v>
+        <v>0.7010999999999999</v>
       </c>
     </row>
     <row r="162">
@@ -19818,7 +19818,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>0.6999</v>
+        <v>0.6991000000000001</v>
       </c>
     </row>
     <row r="163">
@@ -19978,7 +19978,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>0.7209</v>
+        <v>0.7235</v>
       </c>
     </row>
     <row r="171">
@@ -19998,7 +19998,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>0.7544999999999999</v>
+        <v>0.7532</v>
       </c>
     </row>
     <row r="172">
@@ -20018,7 +20018,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>0.7261</v>
+        <v>0.7274</v>
       </c>
     </row>
     <row r="173">
@@ -20038,7 +20038,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>0.6253</v>
+        <v>0.6227</v>
       </c>
     </row>
     <row r="174">
@@ -20058,7 +20058,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>0.7571</v>
+        <v>0.7519</v>
       </c>
     </row>
     <row r="175">
@@ -20078,7 +20078,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>0.6312</v>
+        <v>0.6309</v>
       </c>
     </row>
     <row r="176">
@@ -20098,7 +20098,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>0.673</v>
+        <v>0.6731</v>
       </c>
     </row>
     <row r="177">
@@ -20118,7 +20118,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>0.6568000000000001</v>
+        <v>0.6566</v>
       </c>
     </row>
     <row r="178">
@@ -20138,7 +20138,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>0.5636</v>
+        <v>0.5635</v>
       </c>
     </row>
     <row r="179">
@@ -20158,7 +20158,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>0.721</v>
+        <v>0.7204</v>
       </c>
     </row>
     <row r="180">
@@ -20178,7 +20178,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>0.679</v>
+        <v>0.6786</v>
       </c>
     </row>
     <row r="181">
@@ -20198,7 +20198,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>0.6487000000000001</v>
+        <v>0.6482</v>
       </c>
     </row>
     <row r="182">
@@ -20315,7 +20315,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.1204</v>
+        <v>0.1225</v>
       </c>
     </row>
     <row r="6">
@@ -20335,7 +20335,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.0684</v>
+        <v>0.06950000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -20355,7 +20355,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.1708</v>
+        <v>0.1733</v>
       </c>
     </row>
     <row r="8">
@@ -20375,7 +20375,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.0594</v>
+        <v>0.0588</v>
       </c>
     </row>
     <row r="9">
@@ -20395,7 +20395,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.0113</v>
+        <v>0.0104</v>
       </c>
     </row>
     <row r="10">
@@ -20415,7 +20415,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.1063</v>
+        <v>0.1054</v>
       </c>
     </row>
     <row r="11">
@@ -20435,7 +20435,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.067</v>
+        <v>0.06560000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -20455,7 +20455,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.0249</v>
+        <v>0.0232</v>
       </c>
     </row>
     <row r="13">
@@ -20475,7 +20475,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.1085</v>
+        <v>0.1074</v>
       </c>
     </row>
     <row r="14">
@@ -20495,7 +20495,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.0253</v>
+        <v>0.0249</v>
       </c>
     </row>
     <row r="15">
@@ -20515,7 +20515,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-0.0139</v>
+        <v>-0.0143</v>
       </c>
     </row>
     <row r="16">
@@ -20535,7 +20535,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.0634</v>
+        <v>0.06279999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -20555,7 +20555,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.08409999999999999</v>
+        <v>0.0842</v>
       </c>
     </row>
     <row r="18">
@@ -20575,7 +20575,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.0408</v>
+        <v>0.0406</v>
       </c>
     </row>
     <row r="19">
@@ -20595,7 +20595,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.129</v>
+        <v>0.1294</v>
       </c>
     </row>
     <row r="20">
@@ -20615,7 +20615,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.0345</v>
+        <v>0.0336</v>
       </c>
     </row>
     <row r="21">
@@ -20635,7 +20635,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-0.0046</v>
+        <v>-0.0053</v>
       </c>
     </row>
     <row r="22">
@@ -20655,7 +20655,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.0745</v>
+        <v>0.0737</v>
       </c>
     </row>
     <row r="23">
@@ -20675,7 +20675,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.061</v>
+        <v>0.06370000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -20695,7 +20695,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.0284</v>
+        <v>0.0308</v>
       </c>
     </row>
     <row r="25">
@@ -20715,7 +20715,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.0955</v>
+        <v>0.0983</v>
       </c>
     </row>
     <row r="26">
@@ -20735,7 +20735,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.0417</v>
+        <v>0.0416</v>
       </c>
     </row>
     <row r="27">
@@ -20755,7 +20755,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.0289</v>
+        <v>0.0287</v>
       </c>
     </row>
     <row r="28">
@@ -20775,7 +20775,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.0538</v>
+        <v>0.0539</v>
       </c>
     </row>
     <row r="29">
@@ -20795,7 +20795,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.0193</v>
+        <v>0.0221</v>
       </c>
     </row>
     <row r="30">
@@ -20815,7 +20815,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.0185</v>
+        <v>0.0214</v>
       </c>
     </row>
     <row r="31">
@@ -20835,7 +20835,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.0022</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="32">
@@ -20855,7 +20855,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.0359</v>
+        <v>0.0388</v>
       </c>
     </row>
     <row r="33">
@@ -20875,7 +20875,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.0263</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="34">
@@ -20895,7 +20895,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.0417</v>
+        <v>0.0407</v>
       </c>
     </row>
     <row r="35">
@@ -20915,7 +20915,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.0196</v>
+        <v>0.0181</v>
       </c>
     </row>
     <row r="36">
@@ -20935,7 +20935,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.0668</v>
+        <v>0.06610000000000001</v>
       </c>
     </row>
     <row r="37">
@@ -20975,7 +20975,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.016</v>
+        <v>0.0157</v>
       </c>
     </row>
     <row r="39">
@@ -20995,7 +20995,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.0413</v>
+        <v>0.0412</v>
       </c>
     </row>
     <row r="40">
@@ -21015,7 +21015,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.0129</v>
+        <v>0.0119</v>
       </c>
     </row>
     <row r="41">
@@ -21035,7 +21035,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.0114</v>
+        <v>0.0104</v>
       </c>
     </row>
     <row r="42">
@@ -21055,7 +21055,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>-0.0035</v>
+        <v>-0.0047</v>
       </c>
     </row>
     <row r="43">
@@ -21075,7 +21075,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.027</v>
+        <v>0.0261</v>
       </c>
     </row>
     <row r="44">
@@ -21095,7 +21095,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.1373</v>
+        <v>0.175</v>
       </c>
     </row>
     <row r="45">
@@ -21115,7 +21115,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.0496</v>
+        <v>0.0506</v>
       </c>
     </row>
     <row r="46">
@@ -21135,7 +21135,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.0238</v>
+        <v>0.0245</v>
       </c>
     </row>
     <row r="47">
@@ -21155,7 +21155,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.0769</v>
+        <v>0.078</v>
       </c>
     </row>
     <row r="48">
@@ -21195,7 +21195,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.0154</v>
+        <v>0.0158</v>
       </c>
     </row>
     <row r="50">
@@ -21235,7 +21235,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.021</v>
+        <v>0.0219</v>
       </c>
     </row>
     <row r="52">
@@ -21255,7 +21255,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.0228</v>
+        <v>0.0235</v>
       </c>
     </row>
     <row r="53">
@@ -21275,7 +21275,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.0066</v>
+        <v>0.0072</v>
       </c>
     </row>
     <row r="54">
@@ -21295,7 +21295,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.0393</v>
+        <v>0.0404</v>
       </c>
     </row>
     <row r="55">
@@ -21315,7 +21315,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.0033</v>
+        <v>0.0017</v>
       </c>
     </row>
     <row r="56">
@@ -21335,7 +21335,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.0581</v>
+        <v>0.0586</v>
       </c>
     </row>
     <row r="57">
@@ -21355,7 +21355,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.0175</v>
+        <v>0.0179</v>
       </c>
     </row>
     <row r="58">
@@ -21375,7 +21375,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.09710000000000001</v>
+        <v>0.0984</v>
       </c>
     </row>
     <row r="59">
@@ -21395,7 +21395,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.0183</v>
+        <v>0.0197</v>
       </c>
     </row>
     <row r="60">
@@ -21415,7 +21415,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>-0.0069</v>
+        <v>-0.0047</v>
       </c>
     </row>
     <row r="61">
@@ -21435,7 +21435,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.042</v>
+        <v>0.0434</v>
       </c>
     </row>
     <row r="62">
@@ -21455,7 +21455,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.0397</v>
+        <v>0.0389</v>
       </c>
     </row>
     <row r="63">
@@ -21475,7 +21475,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.0409</v>
+        <v>0.0397</v>
       </c>
     </row>
     <row r="64">
@@ -21495,7 +21495,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.004</v>
+        <v>0.0011</v>
       </c>
     </row>
     <row r="65">
@@ -21515,7 +21515,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.0775</v>
+        <v>0.078</v>
       </c>
     </row>
     <row r="66">
@@ -21535,7 +21535,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.0317</v>
+        <v>0.0453</v>
       </c>
     </row>
     <row r="67">
@@ -21555,7 +21555,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.0253</v>
+        <v>0.0324</v>
       </c>
     </row>
     <row r="68">
@@ -21575,7 +21575,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>-0.018</v>
+        <v>-0.0112</v>
       </c>
     </row>
     <row r="69">
@@ -21595,7 +21595,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.0678</v>
+        <v>0.07530000000000001</v>
       </c>
     </row>
     <row r="70">
@@ -21615,7 +21615,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.015</v>
+        <v>0.0149</v>
       </c>
     </row>
     <row r="71">
@@ -21635,7 +21635,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>-0.0148</v>
+        <v>-0.0139</v>
       </c>
     </row>
     <row r="72">
@@ -21655,7 +21655,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.0436</v>
+        <v>0.0431</v>
       </c>
     </row>
     <row r="73">
@@ -21675,7 +21675,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.0103</v>
+        <v>0.0175</v>
       </c>
     </row>
     <row r="74">
@@ -21695,7 +21695,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.0007</v>
+        <v>0.009299999999999999</v>
       </c>
     </row>
     <row r="75">
@@ -21715,7 +21715,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>-0.0325</v>
+        <v>-0.0211</v>
       </c>
     </row>
     <row r="76">
@@ -21735,7 +21735,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.0335</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="77">
@@ -21755,7 +21755,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.9813</v>
+        <v>0.5423</v>
       </c>
     </row>
     <row r="78">
@@ -21835,7 +21835,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.1292</v>
+        <v>0.1294</v>
       </c>
     </row>
     <row r="82">
@@ -21855,7 +21855,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.137</v>
+        <v>0.1375</v>
       </c>
     </row>
     <row r="83">
@@ -21915,7 +21915,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="86">
@@ -21935,7 +21935,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.2077</v>
+        <v>0.2076</v>
       </c>
     </row>
     <row r="87">
@@ -21955,7 +21955,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.2057</v>
+        <v>0.2205</v>
       </c>
     </row>
     <row r="88">
@@ -22015,7 +22015,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="91">
@@ -22035,7 +22035,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.3099</v>
+        <v>0.3101</v>
       </c>
     </row>
     <row r="92">
@@ -22055,7 +22055,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.2635</v>
+        <v>0.2481</v>
       </c>
     </row>
     <row r="93">
@@ -22135,7 +22135,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.4462</v>
+        <v>0.4464</v>
       </c>
     </row>
     <row r="97">
@@ -22155,7 +22155,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.5085</v>
+        <v>0.5049</v>
       </c>
     </row>
     <row r="98">
@@ -22235,7 +22235,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.618</v>
+        <v>0.6183</v>
       </c>
     </row>
     <row r="102">
@@ -22255,7 +22255,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.6394</v>
+        <v>0.639</v>
       </c>
     </row>
     <row r="103">
@@ -22335,7 +22335,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.1546</v>
+        <v>0.1547</v>
       </c>
     </row>
     <row r="107">
@@ -22435,7 +22435,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.2236</v>
+        <v>0.2237</v>
       </c>
     </row>
     <row r="112">
@@ -22535,7 +22535,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0.3132</v>
+        <v>0.3134</v>
       </c>
     </row>
     <row r="117">
@@ -22635,7 +22635,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>0.4275</v>
+        <v>0.4277</v>
       </c>
     </row>
     <row r="122">
@@ -22735,7 +22735,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>0.5669</v>
+        <v>0.5672</v>
       </c>
     </row>
     <row r="127">
@@ -23095,7 +23095,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>0.164</v>
+        <v>0.1624</v>
       </c>
     </row>
     <row r="145">
@@ -23115,7 +23115,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>0.1444</v>
+        <v>0.1483</v>
       </c>
     </row>
     <row r="146">
@@ -23135,7 +23135,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>0.1222</v>
+        <v>0.1195</v>
       </c>
     </row>
     <row r="147">
@@ -23155,7 +23155,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>0.1356</v>
+        <v>0.1375</v>
       </c>
     </row>
     <row r="148">
@@ -23215,7 +23215,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0.0347</v>
+        <v>0.0419</v>
       </c>
     </row>
     <row r="151">
@@ -23850,7 +23850,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.6992</v>
+        <v>0.7003</v>
       </c>
     </row>
     <row r="9">
@@ -23870,7 +23870,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.6861</v>
+        <v>0.6859</v>
       </c>
     </row>
     <row r="10">
@@ -23890,7 +23890,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.6218</v>
+        <v>0.6219</v>
       </c>
     </row>
     <row r="11">
@@ -23910,7 +23910,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.5658</v>
+        <v>0.5642</v>
       </c>
     </row>
     <row r="12">
@@ -23930,7 +23930,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.6841</v>
+        <v>0.6835</v>
       </c>
     </row>
     <row r="13">
@@ -24034,7 +24034,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.0132</v>
+        <v>0.0144</v>
       </c>
     </row>
     <row r="18">
@@ -24054,7 +24054,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.0135</v>
+        <v>0.0136</v>
       </c>
     </row>
     <row r="19">
@@ -24074,7 +24074,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>-0.0136</v>
+        <v>-0.0124</v>
       </c>
     </row>
     <row r="20">
@@ -24094,7 +24094,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.0396</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="21">
@@ -24114,7 +24114,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.3183</v>
+        <v>0.283</v>
       </c>
     </row>
     <row r="22">
@@ -24176,7 +24176,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.0774</v>
+        <v>0.0784</v>
       </c>
     </row>
     <row r="25">
@@ -24196,7 +24196,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.025</v>
+        <v>0.0249</v>
       </c>
     </row>
     <row r="26">
@@ -24216,7 +24216,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.0284</v>
+        <v>0.0298</v>
       </c>
     </row>
     <row r="27">
@@ -24236,7 +24236,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.1264</v>
+        <v>0.1267</v>
       </c>
     </row>
     <row r="28">
@@ -24318,7 +24318,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.0149</v>
+        <v>0.0166</v>
       </c>
     </row>
     <row r="32">
@@ -24338,7 +24338,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.0146</v>
+        <v>0.0148</v>
       </c>
     </row>
     <row r="33">
@@ -24358,7 +24358,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-0.0134</v>
+        <v>-0.0117</v>
       </c>
     </row>
     <row r="34">
@@ -24378,7 +24378,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.0437</v>
+        <v>0.0461</v>
       </c>
     </row>
     <row r="35">
@@ -24398,7 +24398,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.3057</v>
+        <v>0.2613</v>
       </c>
     </row>
     <row r="36">
@@ -24460,7 +24460,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.0563</v>
+        <v>0.0579</v>
       </c>
     </row>
     <row r="39">
@@ -24480,7 +24480,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.0267</v>
+        <v>0.0266</v>
       </c>
     </row>
     <row r="40">
@@ -24500,7 +24500,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.0042</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="41">
@@ -24520,7 +24520,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.1087</v>
+        <v>0.1098</v>
       </c>
     </row>
     <row r="42">
@@ -24540,7 +24540,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.036</v>
+        <v>0.0307</v>
       </c>
     </row>
     <row r="43">
@@ -24662,7 +24662,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.6892</v>
+        <v>0.6881</v>
       </c>
     </row>
     <row r="49">
@@ -24682,7 +24682,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.6614</v>
+        <v>0.6637999999999999</v>
       </c>
     </row>
     <row r="50">
@@ -24702,7 +24702,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.5686</v>
+        <v>0.5683</v>
       </c>
     </row>
     <row r="51">
@@ -24722,7 +24722,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.4828</v>
+        <v>0.4853</v>
       </c>
     </row>
     <row r="52">
@@ -24742,7 +24742,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.7101</v>
+        <v>0.711</v>
       </c>
     </row>
     <row r="53">
@@ -24846,7 +24846,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.0283</v>
+        <v>0.0248</v>
       </c>
     </row>
     <row r="58">
@@ -24866,7 +24866,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.0225</v>
+        <v>0.0224</v>
       </c>
     </row>
     <row r="59">
@@ -24886,7 +24886,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>-0.0155</v>
+        <v>-0.0192</v>
       </c>
     </row>
     <row r="60">
@@ -24906,7 +24906,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.0723</v>
+        <v>0.06859999999999999</v>
       </c>
     </row>
     <row r="61">
@@ -24926,7 +24926,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.202</v>
+        <v>0.2633</v>
       </c>
     </row>
     <row r="62">
@@ -24988,7 +24988,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.1208</v>
+        <v>0.1201</v>
       </c>
     </row>
     <row r="65">
@@ -25008,7 +25008,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.0354</v>
+        <v>0.0352</v>
       </c>
     </row>
     <row r="66">
@@ -25028,7 +25028,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.0525</v>
+        <v>0.0519</v>
       </c>
     </row>
     <row r="67">
@@ -25048,7 +25048,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.1904</v>
+        <v>0.1897</v>
       </c>
     </row>
     <row r="68">
@@ -25130,7 +25130,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>-0.0211</v>
+        <v>-0.0232</v>
       </c>
     </row>
     <row r="72">
@@ -25150,7 +25150,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.0262</v>
+        <v>0.0263</v>
       </c>
     </row>
     <row r="73">
@@ -25170,7 +25170,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>-0.0727</v>
+        <v>-0.07489999999999999</v>
       </c>
     </row>
     <row r="74">
@@ -25190,7 +25190,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.0296</v>
+        <v>0.0277</v>
       </c>
     </row>
     <row r="75">
@@ -25210,7 +25210,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.4257</v>
+        <v>0.3827</v>
       </c>
     </row>
     <row r="76">
@@ -25272,7 +25272,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08409999999999999</v>
       </c>
     </row>
     <row r="79">
@@ -25292,7 +25292,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.0472</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="80">
@@ -25312,7 +25312,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>-0.0062</v>
+        <v>-0.008699999999999999</v>
       </c>
     </row>
     <row r="81">
@@ -25332,7 +25332,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.1779</v>
+        <v>0.1754</v>
       </c>
     </row>
     <row r="82">
@@ -25352,7 +25352,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.0677</v>
+        <v>0.0747</v>
       </c>
     </row>
     <row r="83">
@@ -25474,7 +25474,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.7141</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="89">
@@ -25494,7 +25494,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.6231</v>
+        <v>0.6247</v>
       </c>
     </row>
     <row r="90">
@@ -25514,7 +25514,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.6898</v>
+        <v>0.6902</v>
       </c>
     </row>
     <row r="91">
@@ -25534,7 +25534,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.469</v>
+        <v>0.4691</v>
       </c>
     </row>
     <row r="92">
@@ -25554,7 +25554,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.6819</v>
+        <v>0.6825</v>
       </c>
     </row>
     <row r="93">
@@ -25658,7 +25658,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.0911</v>
+        <v>0.08939999999999999</v>
       </c>
     </row>
     <row r="98">
@@ -25678,7 +25678,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.0248</v>
+        <v>0.0247</v>
       </c>
     </row>
     <row r="99">
@@ -25698,7 +25698,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.0451</v>
+        <v>0.0437</v>
       </c>
     </row>
     <row r="100">
@@ -25718,7 +25718,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.1449</v>
+        <v>0.1429</v>
       </c>
     </row>
     <row r="101">
@@ -25800,7 +25800,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.0236</v>
+        <v>0.0231</v>
       </c>
     </row>
     <row r="105">
@@ -25840,7 +25840,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>-0.06859999999999999</v>
+        <v>-0.0701</v>
       </c>
     </row>
     <row r="107">
@@ -25860,7 +25860,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.1197</v>
+        <v>0.1192</v>
       </c>
     </row>
     <row r="108">
@@ -25880,7 +25880,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.64</v>
+        <v>0.638</v>
       </c>
     </row>
     <row r="109">
@@ -25942,7 +25942,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.0327</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="112">
@@ -25962,7 +25962,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.0258</v>
+        <v>0.0259</v>
       </c>
     </row>
     <row r="113">
@@ -25982,7 +25982,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>-0.019</v>
+        <v>-0.0202</v>
       </c>
     </row>
     <row r="114">
@@ -26002,7 +26002,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.0805</v>
+        <v>0.0804</v>
       </c>
     </row>
     <row r="115">
@@ -26022,7 +26022,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.212</v>
+        <v>0.2213</v>
       </c>
     </row>
     <row r="116">
@@ -26084,7 +26084,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.2212</v>
+        <v>0.2216</v>
       </c>
     </row>
     <row r="119">
@@ -26104,7 +26104,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.0508</v>
+        <v>0.0505</v>
       </c>
     </row>
     <row r="120">
@@ -26124,7 +26124,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>0.1262</v>
+        <v>0.1272</v>
       </c>
     </row>
     <row r="121">
@@ -26144,7 +26144,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>0.3254</v>
+        <v>0.3259</v>
       </c>
     </row>
     <row r="122">
@@ -26306,7 +26306,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0.6015</v>
+        <v>0.6008</v>
       </c>
     </row>
     <row r="130">
@@ -26346,7 +26346,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0.5027</v>
+        <v>0.5042</v>
       </c>
     </row>
     <row r="132">
@@ -26366,7 +26366,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0.6169</v>
+        <v>0.616</v>
       </c>
     </row>
     <row r="133">
@@ -26470,7 +26470,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.0164</v>
+        <v>0.0172</v>
       </c>
     </row>
     <row r="138">
@@ -26510,7 +26510,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>-0.0181</v>
+        <v>-0.0173</v>
       </c>
     </row>
     <row r="140">
@@ -26530,7 +26530,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>0.0496</v>
+        <v>0.0505</v>
       </c>
     </row>
     <row r="141">
@@ -26550,7 +26550,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>0.3337</v>
+        <v>0.3163</v>
       </c>
     </row>
     <row r="142">
@@ -26612,7 +26612,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>0.0726</v>
+        <v>0.0725</v>
       </c>
     </row>
     <row r="145">
@@ -26692,7 +26692,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0.0073</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="149">
@@ -26754,7 +26754,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>0.0012</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="152">
@@ -26774,7 +26774,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>0.014</v>
+        <v>0.0141</v>
       </c>
     </row>
     <row r="153">
@@ -26794,7 +26794,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>-0.0258</v>
+        <v>-0.025</v>
       </c>
     </row>
     <row r="154">
@@ -26814,7 +26814,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>0.0284</v>
+        <v>0.0296</v>
       </c>
     </row>
     <row r="155">
@@ -26834,7 +26834,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>0.9437</v>
+        <v>0.8943</v>
       </c>
     </row>
     <row r="156">
@@ -26896,7 +26896,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>0.0423</v>
+        <v>0.0408</v>
       </c>
     </row>
     <row r="159">
@@ -26936,7 +26936,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>-0.0265</v>
+        <v>-0.0278</v>
       </c>
     </row>
     <row r="161">
@@ -26956,7 +26956,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0.1113</v>
+        <v>0.1099</v>
       </c>
     </row>
     <row r="162">
@@ -26976,7 +26976,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>0.226</v>
+        <v>0.2417</v>
       </c>
     </row>
     <row r="163">
@@ -27098,7 +27098,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>0.6311</v>
+        <v>0.629</v>
       </c>
     </row>
     <row r="169">
@@ -27118,7 +27118,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>0.6125</v>
+        <v>0.613</v>
       </c>
     </row>
     <row r="170">
@@ -27138,7 +27138,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>0.5819</v>
+        <v>0.5841</v>
       </c>
     </row>
     <row r="171">
@@ -27158,7 +27158,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>0.5358000000000001</v>
+        <v>0.5364</v>
       </c>
     </row>
     <row r="172">
@@ -27282,7 +27282,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>0.0184</v>
+        <v>0.0157</v>
       </c>
     </row>
     <row r="178">
@@ -27302,7 +27302,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>0.0178</v>
+        <v>0.0177</v>
       </c>
     </row>
     <row r="179">
@@ -27322,7 +27322,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>-0.0162</v>
+        <v>-0.0192</v>
       </c>
     </row>
     <row r="180">
@@ -27342,7 +27342,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>0.0529</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="181">
@@ -27362,7 +27362,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>0.2987</v>
+        <v>0.369</v>
       </c>
     </row>
     <row r="182">
@@ -27424,7 +27424,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>0.0495</v>
+        <v>0.0452</v>
       </c>
     </row>
     <row r="185">
@@ -27444,7 +27444,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>0.0315</v>
+        <v>0.0312</v>
       </c>
     </row>
     <row r="186">
@@ -27464,7 +27464,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>-0.0127</v>
+        <v>-0.0155</v>
       </c>
     </row>
     <row r="187">
@@ -27484,7 +27484,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>0.1122</v>
+        <v>0.107</v>
       </c>
     </row>
     <row r="188">
@@ -27504,7 +27504,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>0.113</v>
+        <v>0.1417</v>
       </c>
     </row>
     <row r="189">
@@ -27566,7 +27566,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>0.0203</v>
+        <v>0.0183</v>
       </c>
     </row>
     <row r="192">
@@ -27586,7 +27586,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>0.019</v>
+        <v>0.0189</v>
       </c>
     </row>
     <row r="193">
@@ -27606,7 +27606,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>-0.0169</v>
+        <v>-0.0186</v>
       </c>
     </row>
     <row r="194">
@@ -27626,7 +27626,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>0.0582</v>
+        <v>0.056</v>
       </c>
     </row>
     <row r="195">
@@ -27646,7 +27646,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>0.2757</v>
+        <v>0.3237</v>
       </c>
     </row>
     <row r="196">
@@ -27708,7 +27708,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>0.0457</v>
+        <v>0.0473</v>
       </c>
     </row>
     <row r="199">
@@ -27728,7 +27728,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>0.0327</v>
+        <v>0.0321</v>
       </c>
     </row>
     <row r="200">
@@ -27748,7 +27748,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>-0.0191</v>
+        <v>-0.0167</v>
       </c>
     </row>
     <row r="201">
@@ -27768,7 +27768,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>0.1091</v>
+        <v>0.1096</v>
       </c>
     </row>
     <row r="202">
@@ -27788,7 +27788,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>0.1637</v>
+        <v>0.139</v>
       </c>
     </row>
     <row r="203">
@@ -28045,7 +28045,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.2445</v>
+        <v>0.2443</v>
       </c>
     </row>
     <row r="13">
@@ -28065,7 +28065,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.1924</v>
+        <v>0.1927</v>
       </c>
     </row>
     <row r="14">
@@ -28085,7 +28085,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.4836</v>
+        <v>0.4838</v>
       </c>
     </row>
     <row r="15">
@@ -28105,7 +28105,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1213</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="16">
@@ -28165,7 +28165,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.4959</v>
+        <v>0.4975</v>
       </c>
     </row>
     <row r="19">
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.622</v>
+        <v>0.6214</v>
       </c>
     </row>
     <row r="20">
@@ -28205,7 +28205,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.5952</v>
+        <v>0.5937</v>
       </c>
     </row>
     <row r="21">
@@ -28225,7 +28225,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.6068</v>
+        <v>0.6073</v>
       </c>
     </row>
     <row r="22">
@@ -28305,7 +28305,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.5107</v>
+        <v>0.5103</v>
       </c>
     </row>
     <row r="26">
@@ -28325,7 +28325,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.6271</v>
+        <v>0.6288</v>
       </c>
     </row>
     <row r="27">
@@ -28365,7 +28365,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.6176</v>
+        <v>0.6195000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>4844</v>
+        <v>4845</v>
       </c>
     </row>
     <row r="30">
@@ -28445,7 +28445,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.5319</v>
+        <v>0.532</v>
       </c>
     </row>
     <row r="33">
@@ -28465,7 +28465,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.6361</v>
+        <v>0.6362</v>
       </c>
     </row>
     <row r="34">
@@ -28485,7 +28485,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.5969</v>
+        <v>0.5968</v>
       </c>
     </row>
     <row r="35">
@@ -28505,7 +28505,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.6289</v>
+        <v>0.6294999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -28525,7 +28525,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9695</v>
+        <v>9696</v>
       </c>
     </row>
     <row r="37">
@@ -28585,7 +28585,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.5661</v>
+        <v>0.5662</v>
       </c>
     </row>
     <row r="40">
@@ -28625,7 +28625,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.5873</v>
+        <v>0.5871</v>
       </c>
     </row>
     <row r="42">
@@ -28645,7 +28645,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.6392</v>
+        <v>0.6395999999999999</v>
       </c>
     </row>
     <row r="43">
@@ -28722,7 +28722,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.6637999999999999</v>
+        <v>0.6637</v>
       </c>
     </row>
     <row r="47">
@@ -28742,7 +28742,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.6596</v>
+        <v>0.6595</v>
       </c>
     </row>
     <row r="48">
@@ -28782,7 +28782,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.7</v>
+        <v>0.6997</v>
       </c>
     </row>
     <row r="50">
@@ -29004,7 +29004,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.6997</v>
+        <v>0.6983</v>
       </c>
     </row>
     <row r="61">
@@ -29164,7 +29164,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.6693</v>
+        <v>0.669</v>
       </c>
     </row>
     <row r="69">
@@ -29184,7 +29184,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.6226</v>
+        <v>0.6232</v>
       </c>
     </row>
     <row r="70">

</xml_diff>

<commit_message>
ModRank v1.3.3: corrections after a third review of the A2 build
The GEO screened variant's direction and the same-fold published values are corrected in the
manuscript sources; Figure 7c shows the best value published on the released folds. Ships the tests
of the corrected survival functions (runnable without pytest), the A2 driver, the metric-parity
file and a public copy of GEO amendment 01; README and FOR_REVIEWERS state the A2 values, and
verify_release.py checks the amendments' files and runs the tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper/nc-submission/source_data/SourceData.xlsx
+++ b/paper/nc-submission/source_data/SourceData.xlsx
@@ -23729,7 +23729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D204"/>
+  <dimension ref="A1:D306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27830,6 +27830,2062 @@
       <c r="D204" t="inlineStr">
         <is>
           <t>cases, not comparable pairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/n_cases</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/events</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/clinical_stage_source</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>SurvPath datasets_csv/clinical_data (the DIMAF-file variant used for the headline is bladder-only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/per_seed[0]</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>0.7003</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/per_seed[1]</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>0.7076</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/per_seed[2]</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>0.6979</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/per_seed[3]</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>0.7094</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/per_seed[4]</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>0.7045</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/primary_mean_over_seeds</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>0.7039</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/sd_over_seeds</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>0.0048</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/published/MOAD-FNet</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/published/DIMAF</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>0.679</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/published/APL</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>0.677</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/published/PIBD</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>0.667</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/published/DSCASurv</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>0.646</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/published/OTSurv</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>0.637</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/published/MMP</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>0.635</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/published/SurvPath</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/best_published_any_protocol</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/best_published_verified_folds</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>0.679</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/beats_best_any</t>
+        </is>
+      </c>
+      <c r="D225" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/blca/beats_best_verified</t>
+        </is>
+      </c>
+      <c r="D226" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/n_cases</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/events</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/clinical_stage_source</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>SurvPath datasets_csv/clinical_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/per_seed[0]</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>0.6881</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/per_seed[1]</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>0.6915</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/per_seed[2]</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>0.6997</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/per_seed[3]</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>0.7034</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/per_seed[4]</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>0.7017</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/primary_mean_over_seeds</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>0.6969</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/sd_over_seeds</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>0.0067</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/published/APL</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>0.794</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/published/DSCASurv</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>0.765</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/published/DIMAF</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>0.759</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/published/MMP</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>0.738</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/published/PIBD</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>0.736</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/published/SurvPath</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>0.655</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/best_published_any_protocol</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>0.794</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/best_published_verified_folds</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>0.736</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/beats_best_any</t>
+        </is>
+      </c>
+      <c r="D245" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/brca/beats_best_verified</t>
+        </is>
+      </c>
+      <c r="D246" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/n_cases</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/events</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/clinical_stage_source</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>SurvPath datasets_csv/clinical_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/per_seed[0]</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>0.714</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/per_seed[1]</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>0.7352</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/per_seed[2]</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>0.7333</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/per_seed[3]</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>0.7276</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/per_seed[4]</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>0.7302999999999999</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/primary_mean_over_seeds</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>0.7281</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/sd_over_seeds</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>0.008399999999999999</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/published/DSCASurv</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>0.832</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/published/APL</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/published/PIBD</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>0.768</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/published/SurvPath</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>0.673</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/published/OTSurv</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>0.667</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/published/MMP</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/best_published_any_protocol</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>0.832</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/best_published_verified_folds</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>0.768</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/beats_best_any</t>
+        </is>
+      </c>
+      <c r="D265" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/coadread/beats_best_verified</t>
+        </is>
+      </c>
+      <c r="D266" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/n_cases</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/events</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/clinical_stage_source</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>SurvPath datasets_csv/clinical_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/per_seed[0]</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>0.6179</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/per_seed[1]</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>0.6222</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/per_seed[2]</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>0.6031</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/per_seed[3]</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>0.6075</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/per_seed[4]</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>0.6212</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/primary_mean_over_seeds</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>0.6143999999999999</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/sd_over_seeds</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>0.0086</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/published/DSCASurv</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>0.666</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/published/APL</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>0.653</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/published/PIBD</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/published/SurvPath</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/best_published_any_protocol</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>0.666</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/best_published_verified_folds</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/beats_best_any</t>
+        </is>
+      </c>
+      <c r="D283" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/hnsc/beats_best_verified</t>
+        </is>
+      </c>
+      <c r="D284" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/n_cases</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/events</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/clinical_stage_source</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>SurvPath datasets_csv/clinical_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/per_seed[0]</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>0.629</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/per_seed[1]</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>0.6418</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/per_seed[2]</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>0.6377</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/per_seed[3]</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>0.6489</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/per_seed[4]</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>0.6466</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/primary_mean_over_seeds</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>0.6408</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/sd_over_seeds</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/published/DSCASurv</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>0.698</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/published/APL</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>0.6860000000000001</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/published/PIBD</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>0.6840000000000001</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/published/MMP</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>0.598</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/published/SurvPath</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>0.592</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/best_published_any_protocol</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>0.698</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/best_published_verified_folds</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>0.6840000000000001</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/beats_best_any</t>
+        </is>
+      </c>
+      <c r="D302" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>A_generalisation/cohorts/stad/beats_best_verified</t>
+        </is>
+      </c>
+      <c r="D303" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>A_generalisation/beats_best_verified_in[0]</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>blca</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>A_generalisation/beats_best_any_in[0]</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>blca</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>c_best_published_same_folds</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>experiments/20260817-blca-confirm/results/ablation-generalisation.json</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>A_generalisation/caveat</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>the four non-bladder cohorts use SurvPath's own single `stage` column, because DIMAF publishes split files for bladder only. They are a generalisation arm for the METHOD, not external validation of the bladder number -- there is no held-out bladder cohort anywhere in this benchmark.</t>
         </is>
       </c>
     </row>

</xml_diff>